<commit_message>
feat: support numeric priority in batch import sub-type columns
Sub-type columns (國科會, 教育部配合款1萬) now accept:
- 1, 2, 3... = applied with priority order (1=first choice)
- Y = applied without priority preference
- blank = not applied

Priority-ordered entries are sorted first, then Y entries in column order.
Updated example Excel to demonstrate the new format.
</commit_message>
<xml_diff>
--- a/docs/博士生獎學金_批次匯入範例.xlsx
+++ b/docs/博士生獎學金_批次匯入範例.xlsx
@@ -530,12 +530,12 @@
           <t>P001234</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="I2" s="2" t="n">
         <v>113</v>
       </c>
@@ -576,15 +576,11 @@
           <t>P001234</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="G3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>113</v>
@@ -627,10 +623,8 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="H4" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
@@ -670,10 +664,8 @@
           <t>P001234</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="G5" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
@@ -762,11 +754,11 @@
           <t>P005678</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="G7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
@@ -786,13 +778,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -957,7 +949,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>是否申請國科會（填 Y 表示申請）</t>
+          <t>申請國科會獎學金。填數字表示志願序（1=第一志願），填 Y 表示申請但無偏好，空白表示不申請</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -967,7 +959,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>1 或 Y</t>
         </is>
       </c>
     </row>
@@ -979,7 +971,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>是否申請教育部配合款（填 Y 表示申請）</t>
+          <t>申請教育部配合款。填數字表示志願序（1=第一志願），填 Y 表示申請但無偏好，空白表示不申請</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -989,7 +981,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>2 或 Y</t>
         </is>
       </c>
     </row>
@@ -1034,6 +1026,41 @@
       <c r="D11" t="inlineStr">
         <is>
           <t>交大資工所</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>志願序填寫說明：</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  填 1 = 第一志願（最優先分配）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  填 2 = 第二志願</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  填 Y = 有申請但無偏好（排在有志願序的後面）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  空白 = 不申請該類型</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: remove Y option from sub-type columns, require numeric priority
Sub-type columns now only accept numeric priority (1=first, 2=second).
Y/blank without order is no longer supported — every applied sub-type
must have an explicit priority number.
</commit_message>
<xml_diff>
--- a/docs/博士生獎學金_批次匯入範例.xlsx
+++ b/docs/博士生獎學金_批次匯入範例.xlsx
@@ -706,15 +706,11 @@
           <t>P001234</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="G6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
@@ -949,7 +945,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>申請國科會獎學金。填數字表示志願序（1=第一志願），填 Y 表示申請但無偏好，空白表示不申請</t>
+          <t>填數字表示志願序（1=第一志願，2=第二志願），空白表示不申請</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -959,7 +955,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 或 Y</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -971,7 +967,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>申請教育部配合款。填數字表示志願序（1=第一志願），填 Y 表示申請但無偏好，空白表示不申請</t>
+          <t>填數字表示志願序（1=第一志願，2=第二志願），空白表示不申請</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -981,7 +977,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2 或 Y</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1053,14 +1049,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  填 Y = 有申請但無偏好（排在有志願序的後面）</t>
+          <t xml:space="preserve">  空白 = 不申請該類型</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  空白 = 不申請該類型</t>
+          <t xml:space="preserve">  至少需填寫一個子類型的志願序</t>
         </is>
       </c>
     </row>

</xml_diff>